<commit_message>
add partial edf results
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/fp/gradient_fp_eval_schedulables.xlsx
+++ b/workspace/framework_paper/fp/gradient_fp_eval_schedulables.xlsx
@@ -588,19 +588,19 @@
         <v>0.6473684210526316</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -608,19 +608,19 @@
         <v>0.6684210526315789</v>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
@@ -628,19 +628,19 @@
         <v>0.6894736842105263</v>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -648,19 +648,19 @@
         <v>0.7105263157894737</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13">
@@ -668,19 +668,19 @@
         <v>0.7315789473684211</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
@@ -688,19 +688,19 @@
         <v>0.7526315789473684</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -708,19 +708,19 @@
         <v>0.7736842105263158</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16">
@@ -728,19 +728,19 @@
         <v>0.7947368421052632</v>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -748,19 +748,19 @@
         <v>0.8157894736842105</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -768,19 +768,19 @@
         <v>0.8368421052631578</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19">
@@ -788,19 +788,19 @@
         <v>0.8578947368421053</v>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20">
@@ -808,19 +808,19 @@
         <v>0.8789473684210527</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21">
@@ -828,19 +828,19 @@
         <v>0.9</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>